<commit_message>
Fix streamlit runtime errors and package config
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -538,7 +538,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -712,7 +712,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C86" t="n">

</xml_diff>